<commit_message>
Changed nr. of tests
</commit_message>
<xml_diff>
--- a/test-data/sscData.xlsx
+++ b/test-data/sscData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Chorus Portal Automation_Work\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D284E30-093A-47F3-A1FB-9D59885BFA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A527EE-113D-4795-9965-F3D99353F338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QA" sheetId="1" r:id="rId1"/>
@@ -1112,9 +1112,6 @@
     <t>TestCase89</t>
   </si>
   <si>
-    <t>Ai4P@ssword4</t>
-  </si>
-  <si>
     <t>AI4HR</t>
   </si>
   <si>
@@ -1256,37 +1253,6 @@
   </si>
   <si>
     <t>https://loyalty-qa.app.fielo.com/dx/api/application/v2/objects?object=Sale</t>
-  </si>
-  <si>
-    <t>{
-  "objectTypeID": "SaleCase",
-  "content": {
-    "Origin": "API",
-    "ExternalID": "3aassdsadsad55aa921945595279542051",
-    "SaleChannelCode": "TT01",
-    "PointOfSaleID": "10",
-    "SaleItems": [
-      {
-        "ProductCode": "19529",
-        "Quantity": 1,
-        "TotalAmount":10
-      },
-      {
-        "ProductCode": "19527",
-        "Quantity": 1,
-        "TotalAmount":10
-      },
-      {
-        "ProductCode": "19856",
-        "Quantity": 1,
-        "TotalAmount":10
-      }
-    ],
-    "SaleDateTime": "2025-07-01T10:56:27.066Z",
-    "MemberExternalID": "99691eb263-3573-4be4-90b5-abe027d7b4ec",
-    "StoreCode": "NW-RJ567"
-  }
-}</t>
   </si>
   <si>
     <t>Create Segment</t>
@@ -1506,8 +1472,8 @@
   "objectTypeID": "Store",
   "content": {
     "Origin": "API",
-    "StoreCode": "NW-RJ466",
-    "Name": "Store NW-RJ466",
+    "StoreCode": "NW-RJ470",
+    "Name": "Store NW-RJ470",
     "Description": "Store6 Description",
     "Address": 
       {
@@ -1524,15 +1490,15 @@
   <si>
     <t>{
   "dataViewParameters": {
-    "StoreCode": "NW-RJ466"
+    "StoreCode": "NW-RJ470"
   }
 }</t>
   </si>
   <si>
-    <t>"Store NW-RJ466"</t>
-  </si>
-  <si>
-    <t>{"content":{"Description":"Store4 Description","Name":"Store NW-RJ466","StoreCode":"NW-RJ466","Address":{"Street":"Street1","City":"City1","StateProvince":"State1","PostalCode":"12345","Country":"BRAZIL"},"IsParticipating":true},"pageInstructions":[]}</t>
+    <t>"Store NW-RJ470"</t>
+  </si>
+  <si>
+    <t>{"content":{"Description":"Store4 Description","Name":"Store NW-RJ470","StoreCode":"NW-RJ470","Address":{"Street":"Street1","City":"City1","StateProvince":"State1","PostalCode":"12345","Country":"BRAZIL"},"IsParticipating":true},"pageInstructions":[]}</t>
   </si>
   <si>
     <t>{
@@ -1541,7 +1507,7 @@
     "Origin": "API",
     "Name":"Nuggets",
     "Description":"Nuggets",
-    "ProductCode": "19526",
+    "ProductCode": "19530",
     "Brand": "Burger King",
     "Category": "Snack",
     "Incentivizable":true
@@ -1551,7 +1517,38 @@
   <si>
     <t>{
   "dataViewParameters": {
-    "ProductCode": "19526"
+    "ProductCode": "19530"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "objectTypeID": "SaleCase",
+  "content": {
+    "Origin": "API",
+    "ExternalID": "3aassdsadsad55aa921945595279542051",
+    "SaleChannelCode": "TT01",
+    "PointOfSaleID": "10",
+    "SaleItems": [
+      {
+        "ProductCode": "19530",
+        "Quantity": 1,
+        "TotalAmount":10
+      },
+      {
+        "ProductCode": "19530",
+        "Quantity": 1,
+        "TotalAmount":10
+      },
+      {
+        "ProductCode": "19856",
+        "Quantity": 1,
+        "TotalAmount":10
+      }
+    ],
+    "SaleDateTime": "2025-07-01T10:56:27.066Z",
+    "MemberExternalID": "99691eb263-3573-4be4-90b5-abe027d7b4ec",
+    "StoreCode": "NW-RJ567"
   }
 }</t>
   </si>
@@ -1560,7 +1557,7 @@
     "content": {
         "Name": "Product",
         "Description": "UpdatedDescription",
-        "ProductCode": "19526",
+        "ProductCode": "19530",
         "Brand": "Brand",
         "Category": "Category",
         "Incentivizable": true
@@ -1574,7 +1571,7 @@
   "content": {
     "Origin": "API",
     "Name": "BK Apparel",
-    "ExternalID": "45674",
+    "ExternalID": "45678",
     "RewardType": "stock_control",
     "RewardExpiration": "2025-09-06T04:00:00.000Z",
     "RewardCost": "",
@@ -1585,9 +1582,12 @@
   <si>
     <t>{
   "dataViewParameters": {
-    "ExternalID": "45674"
+    "ExternalID": "45678"
   }
 }</t>
+  </si>
+  <si>
+    <t>Ai4P@ssword5</t>
   </si>
 </sst>
 </file>
@@ -2159,7 +2159,7 @@
         <v>34</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>5</v>
@@ -2185,7 +2185,7 @@
         <v>34</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>5</v>
@@ -2211,7 +2211,7 @@
         <v>34</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>5</v>
@@ -2235,7 +2235,7 @@
         <v>34</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>5</v>
@@ -2283,7 +2283,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>5</v>
@@ -2306,7 +2306,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>5</v>
@@ -2335,7 +2335,7 @@
         <v>34</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="S8" s="6" t="s">
         <v>187</v>
@@ -2352,7 +2352,7 @@
         <v>34</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -2360,7 +2360,7 @@
     <hyperlink ref="H2" r:id="rId1" xr:uid="{C7A33EB6-8367-4005-A814-B19729D1B87B}"/>
     <hyperlink ref="H3" r:id="rId2" xr:uid="{6B0F5573-1B6D-40BD-A1CD-4FF2D6A12B60}"/>
     <hyperlink ref="D2" r:id="rId3" display="Ai4P@ssword3" xr:uid="{BFC9E07A-6B6B-4917-9373-71F733F22D5F}"/>
-    <hyperlink ref="D9" r:id="rId4" display="Ai4P@ssword3" xr:uid="{C693285A-AACF-4030-BAA6-4C6360692518}"/>
+    <hyperlink ref="D9" r:id="rId4" display="Ai4P@ssword4" xr:uid="{C693285A-AACF-4030-BAA6-4C6360692518}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
@@ -5047,7 +5047,7 @@
         <v>34</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" s="10" t="s">
@@ -5063,7 +5063,7 @@
         <v>1</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="M2" s="6" t="s">
         <v>5</v>
@@ -5086,7 +5086,7 @@
         <v>34</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G3" s="8"/>
       <c r="H3" s="6" t="s">
@@ -5125,7 +5125,7 @@
         <v>34</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G4" s="8"/>
       <c r="H4" s="10" t="s">
@@ -5164,7 +5164,7 @@
         <v>34</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G5" s="8"/>
       <c r="H5" s="10" t="s">
@@ -5203,7 +5203,7 @@
         <v>34</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G6" s="8"/>
       <c r="H6" s="10" t="s">
@@ -5242,7 +5242,7 @@
         <v>34</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="10" t="s">
@@ -5281,7 +5281,7 @@
         <v>34</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G8" s="8"/>
       <c r="H8" s="10" t="s">
@@ -5320,7 +5320,7 @@
         <v>34</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="10" t="s">
@@ -5359,7 +5359,7 @@
         <v>34</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G10" s="8"/>
       <c r="H10" s="10" t="s">
@@ -5398,7 +5398,7 @@
         <v>34</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G11" s="8"/>
       <c r="H11" s="10" t="s">
@@ -5437,7 +5437,7 @@
         <v>34</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="10" t="s">
@@ -5476,7 +5476,7 @@
         <v>34</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="10" t="s">
@@ -5515,7 +5515,7 @@
         <v>34</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="10" t="s">
@@ -5554,7 +5554,7 @@
         <v>34</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="10" t="s">
@@ -5593,7 +5593,7 @@
         <v>34</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="10" t="s">
@@ -5632,7 +5632,7 @@
         <v>34</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="10" t="s">
@@ -5671,7 +5671,7 @@
         <v>34</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="10" t="s">
@@ -5710,7 +5710,7 @@
         <v>34</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="10" t="s">
@@ -5749,7 +5749,7 @@
         <v>34</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="10" t="s">
@@ -5788,7 +5788,7 @@
         <v>34</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="10" t="s">
@@ -5827,7 +5827,7 @@
         <v>34</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="10" t="s">
@@ -5866,7 +5866,7 @@
         <v>34</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G23" s="8"/>
       <c r="H23" s="10" t="s">
@@ -5905,7 +5905,7 @@
         <v>34</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G24" s="8"/>
       <c r="H24" s="6" t="s">
@@ -5944,7 +5944,7 @@
         <v>34</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G25" s="8"/>
       <c r="H25" s="10" t="s">
@@ -5983,7 +5983,7 @@
         <v>34</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G26" s="8"/>
       <c r="H26" s="6" t="s">
@@ -6022,7 +6022,7 @@
         <v>34</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="10" t="s">
@@ -6061,7 +6061,7 @@
         <v>34</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="6" t="s">
@@ -6100,7 +6100,7 @@
         <v>34</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="6" t="s">
@@ -6139,7 +6139,7 @@
         <v>34</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G30" s="8"/>
       <c r="H30" s="6" t="s">
@@ -6178,7 +6178,7 @@
         <v>34</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="6" t="s">
@@ -6217,7 +6217,7 @@
         <v>34</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="6" t="s">
@@ -6256,7 +6256,7 @@
         <v>34</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G33" s="8"/>
       <c r="H33" s="6" t="s">
@@ -6295,7 +6295,7 @@
         <v>34</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G34" s="8"/>
       <c r="H34" s="6" t="s">
@@ -6328,7 +6328,7 @@
         <v>34</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="6" t="s">
@@ -6361,7 +6361,7 @@
         <v>34</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G36" s="8"/>
       <c r="H36" s="6" t="s">
@@ -6394,7 +6394,7 @@
         <v>34</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G37" s="8"/>
       <c r="H37" s="6" t="s">
@@ -6427,7 +6427,7 @@
         <v>34</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G38" s="8"/>
       <c r="H38" s="6" t="s">
@@ -6469,7 +6469,7 @@
         <v>34</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="6" t="s">
@@ -6511,7 +6511,7 @@
         <v>34</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="6" t="s">
@@ -6553,7 +6553,7 @@
         <v>34</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="6" t="s">
@@ -6595,7 +6595,7 @@
         <v>34</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="6" t="s">
@@ -6637,7 +6637,7 @@
         <v>34</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G43" s="8"/>
       <c r="L43" s="10" t="s">
@@ -6667,7 +6667,7 @@
         <v>34</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G44" s="8"/>
       <c r="N44" s="6" t="s">
@@ -6691,7 +6691,7 @@
         <v>34</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G45" s="8"/>
       <c r="N45" s="6" t="s">
@@ -6715,7 +6715,7 @@
         <v>34</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G46" s="8"/>
       <c r="N46" s="6" t="s">
@@ -6739,7 +6739,7 @@
         <v>34</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G47" s="8"/>
       <c r="N47" s="6" t="s">
@@ -6763,7 +6763,7 @@
         <v>34</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G48" s="8"/>
       <c r="N48" s="6" t="s">
@@ -6787,7 +6787,7 @@
         <v>34</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G49" s="8"/>
       <c r="N49" s="6" t="s">
@@ -6811,7 +6811,7 @@
         <v>34</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G50" s="8"/>
       <c r="N50" s="6" t="s">
@@ -6835,7 +6835,7 @@
         <v>34</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G51" s="8"/>
       <c r="N51" s="6" t="s">
@@ -6859,7 +6859,7 @@
         <v>34</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G52" s="8"/>
       <c r="N52" s="6" t="s">
@@ -6883,7 +6883,7 @@
         <v>34</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G53" s="8"/>
       <c r="N53" s="6" t="s">
@@ -6907,7 +6907,7 @@
         <v>34</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G54" s="8"/>
       <c r="N54" s="6" t="s">
@@ -6931,7 +6931,7 @@
         <v>34</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G55" s="8"/>
       <c r="N55" s="6" t="s">
@@ -6955,7 +6955,7 @@
         <v>34</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G56" s="8"/>
       <c r="N56" s="6" t="s">
@@ -6979,7 +6979,7 @@
         <v>34</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G57" s="8"/>
       <c r="N57" s="6" t="s">
@@ -7003,7 +7003,7 @@
         <v>34</v>
       </c>
       <c r="F58" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G58" s="8"/>
       <c r="N58" s="6" t="s">
@@ -7027,7 +7027,7 @@
         <v>34</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G59" s="8"/>
       <c r="O59" s="6" t="s">
@@ -7054,7 +7054,7 @@
         <v>34</v>
       </c>
       <c r="F60" s="8" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G60" s="8"/>
       <c r="Q60" s="6" t="s">
@@ -7078,7 +7078,7 @@
         <v>34</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
     </row>
     <row r="62" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
@@ -7098,7 +7098,7 @@
         <v>34</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
     </row>
     <row r="63" spans="1:17" ht="230.4" x14ac:dyDescent="0.3">
@@ -7118,7 +7118,7 @@
         <v>34</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
       <c r="G63" s="20" t="s">
         <v>329</v>
@@ -7141,7 +7141,7 @@
         <v>34</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>333</v>
+        <v>428</v>
       </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.3">
@@ -7899,10 +7899,11 @@
     <hyperlink ref="F56" r:id="rId121" display="Ai4P@ssword3" xr:uid="{71A4E974-AFEB-41B7-8662-9FCF3C37A6E9}"/>
     <hyperlink ref="F57" r:id="rId122" display="Ai4P@ssword3" xr:uid="{A2E209E2-0A14-437E-90BF-8A35B255954E}"/>
     <hyperlink ref="F58" r:id="rId123" display="Ai4P@ssword3" xr:uid="{280D1C2C-2C64-4631-94CB-4C9A63A22A3B}"/>
+    <hyperlink ref="F2" r:id="rId124" display="Ai4P@ssword4" xr:uid="{B5F9DBAD-A1A7-454B-96C6-8035CCE043EB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId124"/>
-  <legacyDrawing r:id="rId125"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId125"/>
+  <legacyDrawing r:id="rId126"/>
 </worksheet>
 </file>
 
@@ -7911,13 +7912,13 @@
   <dimension ref="A1:S72"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.21875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="102.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5546875" style="6" customWidth="1"/>
-    <col min="7" max="8" width="13.88671875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="9.5546875" style="6" hidden="1" customWidth="1"/>
+    <col min="7" max="8" width="13.88671875" style="6" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="34.44140625" style="20" customWidth="1"/>
     <col min="10" max="10" width="21.21875" style="6" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="11.5546875" style="6" hidden="1" customWidth="1"/>
@@ -7925,10 +7926,10 @@
     <col min="13" max="13" width="11.77734375" style="23" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="25.5546875" style="6" customWidth="1"/>
     <col min="15" max="15" width="30.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="28.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.77734375" style="6" customWidth="1"/>
-    <col min="18" max="18" width="11.21875" style="6" customWidth="1"/>
-    <col min="19" max="19" width="10.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.109375" style="6" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="17.77734375" style="6" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="11.21875" style="6" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="10.109375" style="6" hidden="1" customWidth="1"/>
     <col min="20" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
@@ -7943,7 +7944,7 @@
         <v>191</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E1" s="18" t="s">
         <v>50</v>
@@ -7955,7 +7956,7 @@
         <v>1</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="I1" s="17" t="s">
         <v>178</v>
@@ -7999,27 +8000,27 @@
         <v>327</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>345</v>
+      </c>
+      <c r="E2" s="19" t="s">
         <v>338</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>346</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>339</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
       <c r="I2" s="24" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
       <c r="N2" s="6" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="72" x14ac:dyDescent="0.3">
@@ -8030,25 +8031,25 @@
         <v>327</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
       <c r="I3" s="24" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="172.8" x14ac:dyDescent="0.3">
@@ -8059,26 +8060,26 @@
         <v>327</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
       <c r="I4" s="24" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="J4" s="10"/>
       <c r="N4" s="10" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="72" x14ac:dyDescent="0.3">
@@ -8089,26 +8090,26 @@
         <v>327</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
       <c r="I5" s="24" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="J5" s="10"/>
       <c r="N5" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="O5" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="187.2" x14ac:dyDescent="0.3">
@@ -8119,26 +8120,26 @@
         <v>327</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="E6" s="19" t="s">
         <v>356</v>
-      </c>
-      <c r="E6" s="19" t="s">
-        <v>357</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="24" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="J6" s="10"/>
       <c r="N6" s="10" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="O6" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="72" x14ac:dyDescent="0.3">
@@ -8149,26 +8150,26 @@
         <v>327</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="E7" s="19" t="s">
         <v>358</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>359</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
       <c r="I7" s="24" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="J7" s="10"/>
       <c r="N7" t="s">
+        <v>405</v>
+      </c>
+      <c r="O7" t="s">
         <v>407</v>
-      </c>
-      <c r="O7" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="57.6" x14ac:dyDescent="0.3">
@@ -8179,49 +8180,49 @@
         <v>327</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="E8" s="19" t="s">
         <v>365</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>366</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="24" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="J8" s="10"/>
       <c r="N8" s="10" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="O8" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="216" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>327</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="E9" s="19" t="s">
         <v>367</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>368</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
       <c r="I9" s="24" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="J9" s="10"/>
       <c r="N9" s="10"/>
@@ -8229,25 +8230,25 @@
     </row>
     <row r="10" spans="1:19" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>327</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="E10" s="19" t="s">
         <v>369</v>
-      </c>
-      <c r="E10" s="19" t="s">
-        <v>370</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="24" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="J10" s="10"/>
       <c r="N10" s="10"/>
@@ -8255,25 +8256,25 @@
     </row>
     <row r="11" spans="1:19" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>327</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D11" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="E11" s="19" t="s">
         <v>374</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>375</v>
       </c>
       <c r="F11" s="7"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="24" t="s">
-        <v>376</v>
+        <v>424</v>
       </c>
       <c r="J11" s="10"/>
       <c r="N11" s="10"/>
@@ -8287,19 +8288,19 @@
         <v>327</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F12" s="7"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="24" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="J12" s="10"/>
       <c r="N12" s="10"/>
@@ -8313,19 +8314,19 @@
         <v>327</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="F13" s="7"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="24" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="J13" s="10"/>
       <c r="N13" s="10"/>
@@ -8339,19 +8340,19 @@
         <v>327</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="F14" s="7"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="24" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="J14" s="10"/>
       <c r="N14" s="10"/>
@@ -8365,19 +8366,19 @@
         <v>327</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="24" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="N15" s="10"/>
       <c r="O15" s="10"/>
@@ -8387,22 +8388,22 @@
         <v>69</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="F16" s="7"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="24" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="J16" s="10"/>
       <c r="N16" s="10"/>
@@ -8413,22 +8414,22 @@
         <v>70</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="F17" s="7"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="24" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
@@ -8436,22 +8437,22 @@
         <v>71</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="24" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="J18" s="10"/>
     </row>
@@ -8460,22 +8461,22 @@
         <v>72</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="24" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="N19" s="10"/>
     </row>
@@ -8484,22 +8485,22 @@
         <v>73</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D20" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="E20" s="19" t="s">
         <v>352</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>353</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="24" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="N20" s="10"/>
     </row>
@@ -8508,22 +8509,22 @@
         <v>74</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D21" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="E21" s="19" t="s">
         <v>354</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>355</v>
       </c>
       <c r="F21" s="7"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="24" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="N21" s="10"/>
     </row>
@@ -8532,22 +8533,22 @@
         <v>75</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D22" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="E22" s="19" t="s">
         <v>360</v>
-      </c>
-      <c r="E22" s="19" t="s">
-        <v>361</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
       <c r="I22" s="24" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="N22" s="10"/>
     </row>
@@ -8556,22 +8557,22 @@
         <v>76</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D23" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="E23" s="19" t="s">
         <v>363</v>
-      </c>
-      <c r="E23" s="19" t="s">
-        <v>364</v>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
       <c r="I23" s="24" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="N23" s="10"/>
     </row>
@@ -8580,22 +8581,22 @@
         <v>77</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D24" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="E24" s="19" t="s">
         <v>371</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>372</v>
       </c>
       <c r="F24" s="7"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="24" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="N24" s="10"/>
     </row>
@@ -8604,22 +8605,22 @@
         <v>78</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="F25" s="7"/>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="24" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="N25" s="10"/>
     </row>
@@ -8628,22 +8629,22 @@
         <v>79</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="F26" s="7"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="24" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="N26" s="10"/>
     </row>
@@ -9166,17 +9167,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add test data spreadsheet
</commit_message>
<xml_diff>
--- a/test-data/sscData.xlsx
+++ b/test-data/sscData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Chorus Portal Automation_Work\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F2C1FC-EAF7-47A7-8A1A-F1BB81E0335B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDB3C18-3D11-4666-98E6-494450949758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3995" uniqueCount="721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3933" uniqueCount="721">
   <si>
     <t>username</t>
   </si>
@@ -17913,9 +17913,6 @@
       <c r="A3" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C3" s="6" t="s">
         <v>177</v>
       </c>
@@ -17954,9 +17951,6 @@
       <c r="A4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C4" s="6" t="s">
         <v>177</v>
       </c>
@@ -17995,9 +17989,6 @@
       <c r="A5" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C5" s="6" t="s">
         <v>177</v>
       </c>
@@ -18036,9 +18027,6 @@
       <c r="A6" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C6" s="6" t="s">
         <v>177</v>
       </c>
@@ -18077,9 +18065,6 @@
       <c r="A7" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C7" s="6" t="s">
         <v>177</v>
       </c>
@@ -18118,9 +18103,6 @@
       <c r="A8" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C8" s="6" t="s">
         <v>177</v>
       </c>
@@ -18159,9 +18141,6 @@
       <c r="A9" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C9" s="6" t="s">
         <v>177</v>
       </c>
@@ -18200,9 +18179,6 @@
       <c r="A10" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C10" s="6" t="s">
         <v>177</v>
       </c>
@@ -18241,9 +18217,6 @@
       <c r="A11" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C11" s="6" t="s">
         <v>177</v>
       </c>
@@ -18282,9 +18255,6 @@
       <c r="A12" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C12" s="6" t="s">
         <v>177</v>
       </c>
@@ -18323,9 +18293,6 @@
       <c r="A13" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C13" s="6" t="s">
         <v>177</v>
       </c>
@@ -18364,9 +18331,6 @@
       <c r="A14" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C14" s="6" t="s">
         <v>177</v>
       </c>
@@ -18405,9 +18369,6 @@
       <c r="A15" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C15" s="6" t="s">
         <v>177</v>
       </c>
@@ -18446,9 +18407,6 @@
       <c r="A16" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C16" s="6" t="s">
         <v>177</v>
       </c>
@@ -18487,9 +18445,6 @@
       <c r="A17" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C17" s="6" t="s">
         <v>177</v>
       </c>
@@ -18528,9 +18483,6 @@
       <c r="A18" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C18" s="6" t="s">
         <v>177</v>
       </c>
@@ -18569,9 +18521,6 @@
       <c r="A19" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C19" s="6" t="s">
         <v>177</v>
       </c>
@@ -18610,9 +18559,6 @@
       <c r="A20" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C20" s="6" t="s">
         <v>177</v>
       </c>
@@ -18651,9 +18597,6 @@
       <c r="A21" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C21" s="6" t="s">
         <v>177</v>
       </c>
@@ -18692,9 +18635,6 @@
       <c r="A22" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C22" s="6" t="s">
         <v>177</v>
       </c>
@@ -18733,9 +18673,6 @@
       <c r="A23" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C23" s="6" t="s">
         <v>177</v>
       </c>
@@ -18774,9 +18711,6 @@
       <c r="A24" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C24" s="6" t="s">
         <v>177</v>
       </c>
@@ -18814,9 +18748,6 @@
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>177</v>
@@ -18848,9 +18779,6 @@
       <c r="A26" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C26" s="6" t="s">
         <v>177</v>
       </c>
@@ -18881,9 +18809,6 @@
       <c r="A27" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C27" s="6" t="s">
         <v>177</v>
       </c>
@@ -18914,9 +18839,6 @@
       <c r="A28" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C28" s="6" t="s">
         <v>177</v>
       </c>
@@ -18955,9 +18877,6 @@
       <c r="A29" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C29" s="6" t="s">
         <v>177</v>
       </c>
@@ -18996,9 +18915,6 @@
       <c r="A30" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C30" s="6" t="s">
         <v>177</v>
       </c>
@@ -19036,9 +18952,6 @@
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>177</v>
@@ -19070,9 +18983,6 @@
       <c r="A32" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="B32" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C32" s="6" t="s">
         <v>177</v>
       </c>
@@ -19111,9 +19021,6 @@
       <c r="A33" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C33" s="6" t="s">
         <v>177</v>
       </c>
@@ -19151,9 +19058,6 @@
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>177</v>
@@ -19185,9 +19089,6 @@
       <c r="A35" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C35" s="6" t="s">
         <v>177</v>
       </c>
@@ -19225,9 +19126,6 @@
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>177</v>
@@ -19259,9 +19157,6 @@
       <c r="A37" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C37" s="6" t="s">
         <v>177</v>
       </c>
@@ -19300,9 +19195,6 @@
       <c r="A38" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C38" s="6" t="s">
         <v>177</v>
       </c>
@@ -19343,9 +19235,6 @@
       <c r="A39" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C39" s="6" t="s">
         <v>177</v>
       </c>
@@ -19386,9 +19275,6 @@
       <c r="A40" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C40" s="6" t="s">
         <v>177</v>
       </c>
@@ -19429,9 +19315,6 @@
       <c r="A41" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C41" s="6" t="s">
         <v>177</v>
       </c>
@@ -19472,9 +19355,6 @@
       <c r="A42" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C42" s="6" t="s">
         <v>177</v>
       </c>
@@ -19515,9 +19395,6 @@
       <c r="A43" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C43" s="6" t="s">
         <v>178</v>
       </c>
@@ -19557,9 +19434,6 @@
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>179</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>180</v>
@@ -19593,9 +19467,6 @@
       <c r="A45" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="B45" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C45" s="6" t="s">
         <v>177</v>
       </c>
@@ -19628,9 +19499,6 @@
       <c r="A46" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="B46" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C46" s="6" t="s">
         <v>177</v>
       </c>
@@ -19663,9 +19531,6 @@
       <c r="A47" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="B47" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C47" s="6" t="s">
         <v>177</v>
       </c>
@@ -19698,9 +19563,6 @@
       <c r="A48" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="B48" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C48" s="6" t="s">
         <v>177</v>
       </c>
@@ -19733,9 +19595,6 @@
       <c r="A49" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="B49" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C49" s="6" t="s">
         <v>177</v>
       </c>
@@ -19768,9 +19627,6 @@
       <c r="A50" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C50" s="6" t="s">
         <v>177</v>
       </c>
@@ -19811,9 +19667,6 @@
       <c r="A51" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C51" s="6" t="s">
         <v>177</v>
       </c>
@@ -19854,9 +19707,6 @@
       <c r="A52" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="B52" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C52" s="6" t="s">
         <v>177</v>
       </c>
@@ -19896,9 +19746,6 @@
     <row r="53" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>202</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>177</v>
@@ -19932,9 +19779,6 @@
       <c r="A54" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C54" s="6" t="s">
         <v>177</v>
       </c>
@@ -19975,9 +19819,6 @@
       <c r="A55" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C55" s="6" t="s">
         <v>177</v>
       </c>
@@ -20017,9 +19858,6 @@
     <row r="56" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
         <v>205</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>177</v>
@@ -20053,9 +19891,6 @@
       <c r="A57" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="B57" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C57" s="6" t="s">
         <v>177</v>
       </c>
@@ -20096,9 +19931,6 @@
       <c r="A58" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="B58" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C58" s="6" t="s">
         <v>177</v>
       </c>
@@ -20139,9 +19971,6 @@
       <c r="A59" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C59" s="6" t="s">
         <v>177</v>
       </c>
@@ -20186,9 +20015,6 @@
       <c r="A60" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C60" s="6" t="s">
         <v>177</v>
       </c>
@@ -20230,9 +20056,6 @@
       <c r="A61" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C61" s="6" t="s">
         <v>177</v>
       </c>
@@ -20268,9 +20091,6 @@
     <row r="62" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
         <v>211</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>177</v>
@@ -20300,9 +20120,6 @@
       <c r="A63" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>424</v>
-      </c>
       <c r="C63" s="6" t="s">
         <v>324</v>
       </c>
@@ -20341,9 +20158,6 @@
     <row r="64" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>285</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>424</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>177</v>

</xml_diff>

<commit_message>
Add test data spreadsheet with changes
</commit_message>
<xml_diff>
--- a/test-data/sscData.xlsx
+++ b/test-data/sscData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Chorus Portal Automation_Work\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDB3C18-3D11-4666-98E6-494450949758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA2F5A3-511D-420C-BB94-D389CE3A1A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QA" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3933" uniqueCount="721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4065" uniqueCount="751">
   <si>
     <t>username</t>
   </si>
@@ -2510,6 +2510,96 @@
   </si>
   <si>
     <t>Ai4P@ssword6</t>
+  </si>
+  <si>
+    <t>startLoc</t>
+  </si>
+  <si>
+    <t>destLoc</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+  <si>
+    <t>Birmingham</t>
+  </si>
+  <si>
+    <t>Coventry</t>
+  </si>
+  <si>
+    <t>London</t>
+  </si>
+  <si>
+    <t>Bristol</t>
+  </si>
+  <si>
+    <t>stDate</t>
+  </si>
+  <si>
+    <t>endDate</t>
+  </si>
+  <si>
+    <t>18-02-2026</t>
+  </si>
+  <si>
+    <t>19-02-2026</t>
+  </si>
+  <si>
+    <t>20-02-2026</t>
+  </si>
+  <si>
+    <t>trPurpose</t>
+  </si>
+  <si>
+    <t>Business Meeting</t>
+  </si>
+  <si>
+    <t>Leisure</t>
+  </si>
+  <si>
+    <t>Seminar</t>
+  </si>
+  <si>
+    <t>stAirport</t>
+  </si>
+  <si>
+    <t>endAirport</t>
+  </si>
+  <si>
+    <t>Birmingham Airport - BHX</t>
+  </si>
+  <si>
+    <t>Cambridge Airpor - CBG</t>
+  </si>
+  <si>
+    <t>Edinburgh</t>
+  </si>
+  <si>
+    <t>Glasgow</t>
+  </si>
+  <si>
+    <t>Leeds</t>
+  </si>
+  <si>
+    <t>Liverpool</t>
+  </si>
+  <si>
+    <t>Manchester</t>
+  </si>
+  <si>
+    <t>Portsmouth</t>
+  </si>
+  <si>
+    <t>Sheffield</t>
+  </si>
+  <si>
+    <t>Southampton</t>
+  </si>
+  <si>
+    <t>Worthing</t>
+  </si>
+  <si>
+    <t>Leicester</t>
   </si>
 </sst>
 </file>
@@ -2611,7 +2701,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -2677,6 +2767,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2991,37 +3083,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:AA30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="12.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="23.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" style="6" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="11" style="6" customWidth="1"/>
+    <col min="7" max="7" width="10.21875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="20.88671875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="11.21875" style="6" customWidth="1"/>
+    <col min="10" max="10" width="8.21875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="12.109375" style="6" customWidth="1"/>
+    <col min="12" max="12" width="11.44140625" style="6" customWidth="1"/>
+    <col min="13" max="13" width="11.21875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" style="6" customWidth="1"/>
+    <col min="15" max="15" width="12.109375" style="6" customWidth="1"/>
+    <col min="16" max="16" width="13.44140625" style="6" customWidth="1"/>
+    <col min="17" max="17" width="23.109375" style="6" customWidth="1"/>
+    <col min="18" max="18" width="15.109375" style="6" customWidth="1"/>
+    <col min="19" max="19" width="14.5546875" style="6" customWidth="1"/>
     <col min="20" max="20" width="21.77734375" style="6" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="15.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.21875" style="6" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="25" max="16384" width="8.88671875" style="6"/>
+    <col min="22" max="22" width="18.77734375" style="23" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.21875" style="28" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.44140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="23" style="6" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
@@ -3079,8 +3174,32 @@
       <c r="S1" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="T1" s="4" t="s">
+        <v>721</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>722</v>
+      </c>
+      <c r="V1" s="22" t="s">
+        <v>723</v>
+      </c>
+      <c r="W1" s="27" t="s">
+        <v>728</v>
+      </c>
+      <c r="X1" s="27" t="s">
+        <v>729</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>733</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>737</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>12</v>
       </c>
@@ -3106,7 +3225,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>13</v>
       </c>
@@ -3132,7 +3251,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>16</v>
       </c>
@@ -3156,7 +3275,7 @@
       </c>
       <c r="H4" s="8"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
@@ -3204,7 +3323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>31</v>
       </c>
@@ -3227,7 +3346,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>33</v>
       </c>
@@ -3256,7 +3375,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>46</v>
       </c>
@@ -3273,7 +3392,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
         <v>58</v>
       </c>
@@ -3285,6 +3404,291 @@
       </c>
       <c r="D9" s="13" t="s">
         <v>720</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>720</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="8"/>
+      <c r="T10" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="U10" s="6" t="s">
+        <v>727</v>
+      </c>
+      <c r="V10" s="23">
+        <v>195</v>
+      </c>
+      <c r="W10" s="28" t="s">
+        <v>730</v>
+      </c>
+      <c r="X10" s="28" t="s">
+        <v>731</v>
+      </c>
+      <c r="Y10" s="6" t="s">
+        <v>736</v>
+      </c>
+      <c r="Z10" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="AA10" s="6" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>720</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="8"/>
+      <c r="T11" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="U11" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="V11" s="23">
+        <v>217</v>
+      </c>
+      <c r="W11" s="28" t="s">
+        <v>730</v>
+      </c>
+      <c r="X11" s="28" t="s">
+        <v>731</v>
+      </c>
+      <c r="Y11" s="6" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>720</v>
+      </c>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="8"/>
+      <c r="T12" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="U12" s="6" t="s">
+        <v>727</v>
+      </c>
+      <c r="V12" s="23">
+        <v>124</v>
+      </c>
+      <c r="W12" s="28" t="s">
+        <v>731</v>
+      </c>
+      <c r="X12" s="28" t="s">
+        <v>732</v>
+      </c>
+      <c r="Y12" s="6" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="T16" s="4" t="s">
+        <v>721</v>
+      </c>
+      <c r="U16" s="4" t="s">
+        <v>722</v>
+      </c>
+      <c r="V16" s="22" t="s">
+        <v>723</v>
+      </c>
+      <c r="W16" s="4" t="s">
+        <v>737</v>
+      </c>
+      <c r="X16" s="4" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="17" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T17" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="U17" s="6" t="s">
+        <v>727</v>
+      </c>
+      <c r="V17" s="23">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T18" s="6" t="s">
+        <v>727</v>
+      </c>
+      <c r="U18" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="V18" s="23">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T19" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="U19" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="V19" s="23">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="20" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T20" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="U20" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="V20" s="23">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T21" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="U21" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="V21" s="23">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="22" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T22" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="U22" t="s">
+        <v>750</v>
+      </c>
+      <c r="V22" s="23">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="23" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T23" t="s">
+        <v>750</v>
+      </c>
+      <c r="U23" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="V23" s="23">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T24" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="U24" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="V24" s="23">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="25" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T25" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="U25" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="V25" s="23">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="26" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T26" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="U26" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="V26" s="23">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="27" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T27" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="U27" s="6" t="s">
+        <v>747</v>
+      </c>
+      <c r="V27" s="23">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="28" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T28" s="6" t="s">
+        <v>747</v>
+      </c>
+      <c r="U28" s="6" t="s">
+        <v>748</v>
+      </c>
+      <c r="V28" s="23">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="29" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T29" s="6" t="s">
+        <v>748</v>
+      </c>
+      <c r="U29" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="V29" s="23">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="30" spans="20:22" x14ac:dyDescent="0.3">
+      <c r="T30" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="U30" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="V30" s="23">
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -3293,9 +3697,12 @@
     <hyperlink ref="H3" r:id="rId2" xr:uid="{6B0F5573-1B6D-40BD-A1CD-4FF2D6A12B60}"/>
     <hyperlink ref="D2" r:id="rId3" display="Ai4P@ssword3" xr:uid="{BFC9E07A-6B6B-4917-9373-71F733F22D5F}"/>
     <hyperlink ref="D9" r:id="rId4" display="Ai4P@ssword4" xr:uid="{C693285A-AACF-4030-BAA6-4C6360692518}"/>
+    <hyperlink ref="D10" r:id="rId5" display="Ai4P@ssword3" xr:uid="{B1AC8471-FE38-491F-AAB3-B38C4048CD41}"/>
+    <hyperlink ref="D11" r:id="rId6" display="Ai4P@ssword3" xr:uid="{ACA9CCDE-DEF1-46AD-B314-6DAEDD9FF34D}"/>
+    <hyperlink ref="D12" r:id="rId7" display="Ai4P@ssword3" xr:uid="{935C9AFC-698F-410C-A364-D9F348F9314C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
 
@@ -17800,7 +18207,8 @@
     <col min="4" max="4" width="7.21875" style="6" customWidth="1"/>
     <col min="5" max="5" width="102.44140625" style="20" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.5546875" style="6" customWidth="1"/>
-    <col min="7" max="8" width="13.88671875" style="6" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" style="6" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="13.88671875" style="6" customWidth="1"/>
     <col min="9" max="10" width="14.109375" style="20" customWidth="1"/>
     <col min="11" max="11" width="11.77734375" style="23" customWidth="1"/>
     <col min="12" max="12" width="25.5546875" style="6" customWidth="1"/>
@@ -17913,6 +18321,9 @@
       <c r="A3" s="6" t="s">
         <v>57</v>
       </c>
+      <c r="B3" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C3" s="6" t="s">
         <v>177</v>
       </c>
@@ -17951,6 +18362,9 @@
       <c r="A4" s="6" t="s">
         <v>64</v>
       </c>
+      <c r="B4" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C4" s="6" t="s">
         <v>177</v>
       </c>
@@ -17989,6 +18403,9 @@
       <c r="A5" s="6" t="s">
         <v>66</v>
       </c>
+      <c r="B5" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C5" s="6" t="s">
         <v>177</v>
       </c>
@@ -18027,6 +18444,9 @@
       <c r="A6" s="6" t="s">
         <v>67</v>
       </c>
+      <c r="B6" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C6" s="6" t="s">
         <v>177</v>
       </c>
@@ -18065,6 +18485,9 @@
       <c r="A7" s="6" t="s">
         <v>68</v>
       </c>
+      <c r="B7" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C7" s="6" t="s">
         <v>177</v>
       </c>
@@ -18103,6 +18526,9 @@
       <c r="A8" s="6" t="s">
         <v>69</v>
       </c>
+      <c r="B8" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C8" s="6" t="s">
         <v>177</v>
       </c>
@@ -18141,6 +18567,9 @@
       <c r="A9" s="6" t="s">
         <v>70</v>
       </c>
+      <c r="B9" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C9" s="6" t="s">
         <v>177</v>
       </c>
@@ -18179,6 +18608,9 @@
       <c r="A10" s="6" t="s">
         <v>71</v>
       </c>
+      <c r="B10" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C10" s="6" t="s">
         <v>177</v>
       </c>
@@ -18217,6 +18649,9 @@
       <c r="A11" s="6" t="s">
         <v>72</v>
       </c>
+      <c r="B11" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C11" s="6" t="s">
         <v>177</v>
       </c>
@@ -18255,6 +18690,9 @@
       <c r="A12" s="6" t="s">
         <v>73</v>
       </c>
+      <c r="B12" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C12" s="6" t="s">
         <v>177</v>
       </c>
@@ -18293,6 +18731,9 @@
       <c r="A13" s="6" t="s">
         <v>74</v>
       </c>
+      <c r="B13" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C13" s="6" t="s">
         <v>177</v>
       </c>
@@ -18331,6 +18772,9 @@
       <c r="A14" s="6" t="s">
         <v>75</v>
       </c>
+      <c r="B14" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C14" s="6" t="s">
         <v>177</v>
       </c>
@@ -18369,6 +18813,9 @@
       <c r="A15" s="6" t="s">
         <v>76</v>
       </c>
+      <c r="B15" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C15" s="6" t="s">
         <v>177</v>
       </c>
@@ -18407,6 +18854,9 @@
       <c r="A16" s="6" t="s">
         <v>77</v>
       </c>
+      <c r="B16" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C16" s="6" t="s">
         <v>177</v>
       </c>
@@ -18445,6 +18895,9 @@
       <c r="A17" s="6" t="s">
         <v>78</v>
       </c>
+      <c r="B17" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C17" s="6" t="s">
         <v>177</v>
       </c>
@@ -18483,6 +18936,9 @@
       <c r="A18" s="6" t="s">
         <v>79</v>
       </c>
+      <c r="B18" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C18" s="6" t="s">
         <v>177</v>
       </c>
@@ -18521,6 +18977,9 @@
       <c r="A19" s="6" t="s">
         <v>80</v>
       </c>
+      <c r="B19" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C19" s="6" t="s">
         <v>177</v>
       </c>
@@ -18559,6 +19018,9 @@
       <c r="A20" s="6" t="s">
         <v>81</v>
       </c>
+      <c r="B20" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C20" s="6" t="s">
         <v>177</v>
       </c>
@@ -18597,6 +19059,9 @@
       <c r="A21" s="6" t="s">
         <v>82</v>
       </c>
+      <c r="B21" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C21" s="6" t="s">
         <v>177</v>
       </c>
@@ -18635,6 +19100,9 @@
       <c r="A22" s="6" t="s">
         <v>83</v>
       </c>
+      <c r="B22" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C22" s="6" t="s">
         <v>177</v>
       </c>
@@ -18673,6 +19141,9 @@
       <c r="A23" s="6" t="s">
         <v>84</v>
       </c>
+      <c r="B23" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C23" s="6" t="s">
         <v>177</v>
       </c>
@@ -18711,6 +19182,9 @@
       <c r="A24" s="6" t="s">
         <v>112</v>
       </c>
+      <c r="B24" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C24" s="6" t="s">
         <v>177</v>
       </c>
@@ -18748,6 +19222,9 @@
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>113</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>177</v>
@@ -18779,6 +19256,9 @@
       <c r="A26" s="6" t="s">
         <v>114</v>
       </c>
+      <c r="B26" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C26" s="6" t="s">
         <v>177</v>
       </c>
@@ -18809,6 +19289,9 @@
       <c r="A27" s="6" t="s">
         <v>115</v>
       </c>
+      <c r="B27" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C27" s="6" t="s">
         <v>177</v>
       </c>
@@ -18839,6 +19322,9 @@
       <c r="A28" s="6" t="s">
         <v>116</v>
       </c>
+      <c r="B28" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C28" s="6" t="s">
         <v>177</v>
       </c>
@@ -18877,6 +19363,9 @@
       <c r="A29" s="6" t="s">
         <v>117</v>
       </c>
+      <c r="B29" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C29" s="6" t="s">
         <v>177</v>
       </c>
@@ -18915,6 +19404,9 @@
       <c r="A30" s="6" t="s">
         <v>118</v>
       </c>
+      <c r="B30" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C30" s="6" t="s">
         <v>177</v>
       </c>
@@ -18952,6 +19444,9 @@
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>119</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>177</v>
@@ -18983,6 +19478,9 @@
       <c r="A32" s="6" t="s">
         <v>120</v>
       </c>
+      <c r="B32" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C32" s="6" t="s">
         <v>177</v>
       </c>
@@ -19021,6 +19519,9 @@
       <c r="A33" s="6" t="s">
         <v>121</v>
       </c>
+      <c r="B33" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C33" s="6" t="s">
         <v>177</v>
       </c>
@@ -19058,6 +19559,9 @@
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>122</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>177</v>
@@ -19089,6 +19593,9 @@
       <c r="A35" s="6" t="s">
         <v>123</v>
       </c>
+      <c r="B35" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C35" s="6" t="s">
         <v>177</v>
       </c>
@@ -19126,6 +19633,9 @@
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>124</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>177</v>
@@ -19157,6 +19667,9 @@
       <c r="A37" s="6" t="s">
         <v>125</v>
       </c>
+      <c r="B37" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C37" s="6" t="s">
         <v>177</v>
       </c>
@@ -19195,6 +19708,9 @@
       <c r="A38" s="6" t="s">
         <v>126</v>
       </c>
+      <c r="B38" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C38" s="6" t="s">
         <v>177</v>
       </c>
@@ -19235,6 +19751,9 @@
       <c r="A39" s="6" t="s">
         <v>127</v>
       </c>
+      <c r="B39" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C39" s="6" t="s">
         <v>177</v>
       </c>
@@ -19275,6 +19794,9 @@
       <c r="A40" s="6" t="s">
         <v>128</v>
       </c>
+      <c r="B40" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C40" s="6" t="s">
         <v>177</v>
       </c>
@@ -19315,6 +19837,9 @@
       <c r="A41" s="6" t="s">
         <v>129</v>
       </c>
+      <c r="B41" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C41" s="6" t="s">
         <v>177</v>
       </c>
@@ -19355,6 +19880,9 @@
       <c r="A42" s="6" t="s">
         <v>165</v>
       </c>
+      <c r="B42" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C42" s="6" t="s">
         <v>177</v>
       </c>
@@ -19395,6 +19923,9 @@
       <c r="A43" s="6" t="s">
         <v>166</v>
       </c>
+      <c r="B43" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C43" s="6" t="s">
         <v>178</v>
       </c>
@@ -19434,6 +19965,9 @@
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>179</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>180</v>
@@ -19467,6 +20001,9 @@
       <c r="A45" s="6" t="s">
         <v>181</v>
       </c>
+      <c r="B45" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C45" s="6" t="s">
         <v>177</v>
       </c>
@@ -19499,6 +20036,9 @@
       <c r="A46" s="6" t="s">
         <v>193</v>
       </c>
+      <c r="B46" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C46" s="6" t="s">
         <v>177</v>
       </c>
@@ -19531,6 +20071,9 @@
       <c r="A47" s="6" t="s">
         <v>196</v>
       </c>
+      <c r="B47" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C47" s="6" t="s">
         <v>177</v>
       </c>
@@ -19563,6 +20106,9 @@
       <c r="A48" s="6" t="s">
         <v>197</v>
       </c>
+      <c r="B48" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C48" s="6" t="s">
         <v>177</v>
       </c>
@@ -19595,6 +20141,9 @@
       <c r="A49" s="6" t="s">
         <v>198</v>
       </c>
+      <c r="B49" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C49" s="6" t="s">
         <v>177</v>
       </c>
@@ -19627,6 +20176,9 @@
       <c r="A50" s="6" t="s">
         <v>199</v>
       </c>
+      <c r="B50" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C50" s="6" t="s">
         <v>177</v>
       </c>
@@ -19667,6 +20219,9 @@
       <c r="A51" s="6" t="s">
         <v>200</v>
       </c>
+      <c r="B51" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C51" s="6" t="s">
         <v>177</v>
       </c>
@@ -19707,6 +20262,9 @@
       <c r="A52" s="6" t="s">
         <v>201</v>
       </c>
+      <c r="B52" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C52" s="6" t="s">
         <v>177</v>
       </c>
@@ -19746,6 +20304,9 @@
     <row r="53" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>202</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>177</v>
@@ -19779,6 +20340,9 @@
       <c r="A54" s="6" t="s">
         <v>203</v>
       </c>
+      <c r="B54" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C54" s="6" t="s">
         <v>177</v>
       </c>
@@ -19819,6 +20383,9 @@
       <c r="A55" s="6" t="s">
         <v>204</v>
       </c>
+      <c r="B55" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C55" s="6" t="s">
         <v>177</v>
       </c>
@@ -19858,6 +20425,9 @@
     <row r="56" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
         <v>205</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>177</v>
@@ -19891,6 +20461,9 @@
       <c r="A57" s="6" t="s">
         <v>206</v>
       </c>
+      <c r="B57" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C57" s="6" t="s">
         <v>177</v>
       </c>
@@ -19931,6 +20504,9 @@
       <c r="A58" s="6" t="s">
         <v>207</v>
       </c>
+      <c r="B58" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C58" s="6" t="s">
         <v>177</v>
       </c>
@@ -19971,6 +20547,9 @@
       <c r="A59" s="6" t="s">
         <v>208</v>
       </c>
+      <c r="B59" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C59" s="6" t="s">
         <v>177</v>
       </c>
@@ -20015,6 +20594,9 @@
       <c r="A60" s="6" t="s">
         <v>209</v>
       </c>
+      <c r="B60" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C60" s="6" t="s">
         <v>177</v>
       </c>
@@ -20056,6 +20638,9 @@
       <c r="A61" s="6" t="s">
         <v>210</v>
       </c>
+      <c r="B61" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C61" s="6" t="s">
         <v>177</v>
       </c>
@@ -20091,6 +20676,9 @@
     <row r="62" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
         <v>211</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>177</v>
@@ -20120,6 +20708,9 @@
       <c r="A63" s="6" t="s">
         <v>274</v>
       </c>
+      <c r="B63" s="6" t="s">
+        <v>424</v>
+      </c>
       <c r="C63" s="6" t="s">
         <v>324</v>
       </c>
@@ -20158,6 +20749,9 @@
     <row r="64" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>285</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>424</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>177</v>

</xml_diff>

<commit_message>
Updated test data file
</commit_message>
<xml_diff>
--- a/test-data/sscData.xlsx
+++ b/test-data/sscData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Chorus Portal Automation_Work\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA2F5A3-511D-420C-BB94-D389CE3A1A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D90AE950-3A88-4C78-B3AB-111650657890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QA" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4065" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4065" uniqueCount="753">
   <si>
     <t>username</t>
   </si>
@@ -2539,15 +2539,6 @@
     <t>endDate</t>
   </si>
   <si>
-    <t>18-02-2026</t>
-  </si>
-  <si>
-    <t>19-02-2026</t>
-  </si>
-  <si>
-    <t>20-02-2026</t>
-  </si>
-  <si>
     <t>trPurpose</t>
   </si>
   <si>
@@ -2569,9 +2560,6 @@
     <t>Birmingham Airport - BHX</t>
   </si>
   <si>
-    <t>Cambridge Airpor - CBG</t>
-  </si>
-  <si>
     <t>Edinburgh</t>
   </si>
   <si>
@@ -2600,6 +2588,24 @@
   </si>
   <si>
     <t>Leicester</t>
+  </si>
+  <si>
+    <t>23-02-2026</t>
+  </si>
+  <si>
+    <t>25-02-2026</t>
+  </si>
+  <si>
+    <t>24-02-2026</t>
+  </si>
+  <si>
+    <t>26-02-2026</t>
+  </si>
+  <si>
+    <t>27-02-2026</t>
+  </si>
+  <si>
+    <t>Cambridge Airport - CBG</t>
   </si>
 </sst>
 </file>
@@ -3111,8 +3117,8 @@
     <col min="23" max="23" width="20.21875" style="28" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="15.44140625" style="28" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="15.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="23" style="6" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="24" style="6" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="28" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
@@ -3190,13 +3196,13 @@
         <v>729</v>
       </c>
       <c r="Y1" s="4" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="Z1" s="4" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="AA1" s="4" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
@@ -3424,28 +3430,28 @@
       <c r="G10" s="7"/>
       <c r="H10" s="8"/>
       <c r="T10" s="6" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="U10" s="6" t="s">
         <v>727</v>
       </c>
       <c r="V10" s="23">
-        <v>195</v>
+        <v>124</v>
       </c>
       <c r="W10" s="28" t="s">
-        <v>730</v>
+        <v>747</v>
       </c>
       <c r="X10" s="28" t="s">
-        <v>731</v>
+        <v>748</v>
       </c>
       <c r="Y10" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="Z10" s="6" t="s">
         <v>736</v>
       </c>
-      <c r="Z10" s="6" t="s">
-        <v>739</v>
-      </c>
       <c r="AA10" s="6" t="s">
-        <v>740</v>
+        <v>752</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.3">
@@ -3466,22 +3472,22 @@
       <c r="G11" s="7"/>
       <c r="H11" s="8"/>
       <c r="T11" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="U11" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="V11" s="23">
+        <v>308</v>
+      </c>
+      <c r="W11" s="28" t="s">
         <v>749</v>
       </c>
-      <c r="U11" s="6" t="s">
-        <v>724</v>
-      </c>
-      <c r="V11" s="23">
-        <v>217</v>
-      </c>
-      <c r="W11" s="28" t="s">
-        <v>730</v>
-      </c>
       <c r="X11" s="28" t="s">
+        <v>750</v>
+      </c>
+      <c r="Y11" s="6" t="s">
         <v>731</v>
-      </c>
-      <c r="Y11" s="6" t="s">
-        <v>734</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.3">
@@ -3502,22 +3508,22 @@
       <c r="G12" s="7"/>
       <c r="H12" s="8"/>
       <c r="T12" s="6" t="s">
-        <v>724</v>
+        <v>742</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>727</v>
+        <v>743</v>
       </c>
       <c r="V12" s="23">
-        <v>124</v>
+        <v>347</v>
       </c>
       <c r="W12" s="28" t="s">
-        <v>731</v>
+        <v>748</v>
       </c>
       <c r="X12" s="28" t="s">
+        <v>751</v>
+      </c>
+      <c r="Y12" s="6" t="s">
         <v>732</v>
-      </c>
-      <c r="Y12" s="6" t="s">
-        <v>735</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
@@ -3531,10 +3537,10 @@
         <v>723</v>
       </c>
       <c r="W16" s="4" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
     </row>
     <row r="17" spans="20:22" x14ac:dyDescent="0.3">
@@ -3564,7 +3570,7 @@
         <v>725</v>
       </c>
       <c r="U19" s="6" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="V19" s="23">
         <v>410</v>
@@ -3572,10 +3578,10 @@
     </row>
     <row r="20" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T20" s="6" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="U20" s="6" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="V20" s="23">
         <v>75</v>
@@ -3583,10 +3589,10 @@
     </row>
     <row r="21" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T21" s="6" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="U21" s="6" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="V21" s="23">
         <v>290</v>
@@ -3594,10 +3600,10 @@
     </row>
     <row r="22" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T22" s="6" t="s">
-        <v>743</v>
+        <v>739</v>
       </c>
       <c r="U22" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="V22" s="23">
         <v>132</v>
@@ -3605,10 +3611,10 @@
     </row>
     <row r="23" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T23" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="U23" s="6" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="V23" s="23">
         <v>150</v>
@@ -3616,7 +3622,7 @@
     </row>
     <row r="24" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T24" s="6" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="U24" s="6" t="s">
         <v>726</v>
@@ -3630,7 +3636,7 @@
         <v>726</v>
       </c>
       <c r="U25" s="6" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="V25" s="23">
         <v>262</v>
@@ -3638,10 +3644,10 @@
     </row>
     <row r="26" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T26" s="6" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="U26" s="6" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="V26" s="23">
         <v>308</v>
@@ -3649,10 +3655,10 @@
     </row>
     <row r="27" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T27" s="6" t="s">
-        <v>746</v>
+        <v>742</v>
       </c>
       <c r="U27" s="6" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="V27" s="23">
         <v>347</v>
@@ -3660,10 +3666,10 @@
     </row>
     <row r="28" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T28" s="6" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="U28" s="6" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="V28" s="23">
         <v>310</v>
@@ -3671,10 +3677,10 @@
     </row>
     <row r="29" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T29" s="6" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="U29" s="6" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="V29" s="23">
         <v>90</v>
@@ -3682,7 +3688,7 @@
     </row>
     <row r="30" spans="20:22" x14ac:dyDescent="0.3">
       <c r="T30" s="6" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="U30" s="6" t="s">
         <v>724</v>

</xml_diff>